<commit_message>
Record O'Neal plus-7 on batch 722; finish in-gate rounding to Success.
Entered 10174–10180 (only seven Aug 1+ bills remained). 10160–10164 untouched.
Anthony plain Comments_1 on missing_receipt 10175/10178. Posted rounding PPV
on 10176/10179/10180 and returned the last two from Transfer AP to 722.
Parent Outlook stays Entered with issues (NOTE-51 siblings not all Success).

Co-authored-by: beave89atm <beave89atm@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/runs/AP-run-2026-09-21-oneal.xlsx
+++ b/runs/AP-run-2026-09-21-oneal.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Exception counts" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'AP run'!$A$1:$Q$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'AP run'!$A$1:$Q$13</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q6"/>
+  <dimension ref="A1:Q13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -944,8 +944,521 @@
       </c>
       <c r="Q6" s="2" t="inlineStr"/>
     </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>O'Neal Steel - Dallas (GP)</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>15460544</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>58920</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>64.5</v>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>Success</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Finished bill (Invoice_Type 3). Header PO set=58920. Select Receipts 23730 240@0.2688 on PO 58920. Invoice #=15460544 (exact PDF). Fees=none (Additional Charge Fees id 11, not missing merch lines / not PPV). PPV=none. Attach status=attached. Finish Select Receipts selected ids=[23730] fees=none ppv=none. Flag status=entered-in-ai.</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr"/>
+      <c r="I7" s="2" t="inlineStr"/>
+      <c r="J7" s="2" t="n">
+        <v>10174</v>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>API Agent - 9/21/26 O'Neal (722)</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="N7" s="2" t="inlineStr">
+        <is>
+          <t>attached</t>
+        </is>
+      </c>
+      <c r="O7" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P7" s="2" t="inlineStr">
+        <is>
+          <t>entered-with-issues</t>
+        </is>
+      </c>
+      <c r="Q7" s="2" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>O'Neal Steel - Dallas (GP)</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>15460995</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>59085</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>6954.21</v>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>category=missing_receipt; owner=Anthony. HOLD (receipt): no open receipt leftover on PO 59085 for O'Neal invoice #15460995. Do not first-open guess. Anthony: receiving must receive the PO so AP can Select Receipts. Comments_1 names Anthony (mention-id unproven). Do not Transfer AP. Outlook AI HOLD. Flag status=entered-with-issues. Comments_1 missing_receipt status=added tab=Comments tab persisted Anthony (list Comments_1 item 929, plain text (no mention-node)). User-alert/notify API not confirmed — dedicated GET comments/mentions/notifications are 404. Header Comments string is the wrong surface and is ignored. transfer_ap=False mention_id=None owner=Anthony mail_send=False.</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>missing_receipt</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>Anthony</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="n">
+        <v>10175</v>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>API Agent - 9/21/26 O'Neal (722)</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="N8" s="2" t="inlineStr">
+        <is>
+          <t>attached</t>
+        </is>
+      </c>
+      <c r="O8" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P8" s="2" t="inlineStr">
+        <is>
+          <t>entered-with-issues</t>
+        </is>
+      </c>
+      <c r="Q8" s="2" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>O'Neal Steel - Dallas (GP)</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>15461007</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>59086</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>67.38</v>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>Success</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Finished bill (Invoice_Type 3). Header PO set=59086. Select Receipts already-selected on PO 59086. Invoice #=15461007 (exact PDF). Amount=67.38 after rounding PPV +0.18. Fees=none. Attach status=attached. Flag status=entered-with-issues (parent siblings not all Success).</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr"/>
+      <c r="I9" s="2" t="inlineStr"/>
+      <c r="J9" s="2" t="n">
+        <v>10176</v>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>API Agent - 9/21/26 O'Neal (722)</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>0.18</t>
+        </is>
+      </c>
+      <c r="N9" s="2" t="inlineStr">
+        <is>
+          <t>attached</t>
+        </is>
+      </c>
+      <c r="O9" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P9" s="2" t="inlineStr">
+        <is>
+          <t>entered-with-issues</t>
+        </is>
+      </c>
+      <c r="Q9" s="2" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>O'Neal Steel - Dallas (GP)</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>15461157</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>59092</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="n">
+        <v>1978.91</v>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>Success</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Finished bill (Invoice_Type 3). Header PO set=59092. Select Receipts 23799 4@494.7275 on PO 59092. Invoice #=15461157 (exact PDF). Fees=none (Additional Charge Fees id 11, not missing merch lines / not PPV). PPV=none. Attach status=attached. Flag status=entered-in-ai.</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr"/>
+      <c r="I10" s="2" t="inlineStr"/>
+      <c r="J10" s="2" t="n">
+        <v>10177</v>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>API Agent - 9/21/26 O'Neal (722)</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="N10" s="2" t="inlineStr">
+        <is>
+          <t>attached</t>
+        </is>
+      </c>
+      <c r="O10" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P10" s="2" t="inlineStr">
+        <is>
+          <t>entered-with-issues</t>
+        </is>
+      </c>
+      <c r="Q10" s="2" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>O'Neal Steel - Dallas (GP)</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>15476365</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>59070</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="n">
+        <v>1115.68</v>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>category=missing_receipt; owner=Anthony. HOLD (receipt): no open receipt leftover on PO 59070 for O'Neal invoice #15476365. Do not first-open guess. Anthony: receiving must receive the PO so AP can Select Receipts. Comments_1 names Anthony (mention-id unproven). Do not Transfer AP. Outlook AI HOLD. Flag status=entered-with-issues. Comments_1 missing_receipt status=added tab=Comments tab persisted Anthony (list Comments_1 item 930, plain text (no mention-node)). User-alert/notify API not confirmed — dedicated GET comments/mentions/notifications are 404. Header Comments string is the wrong surface and is ignored. transfer_ap=False mention_id=None owner=Anthony mail_send=False.</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>missing_receipt</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>Anthony</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="n">
+        <v>10178</v>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>API Agent - 9/21/26 O'Neal (722)</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="N11" s="2" t="inlineStr">
+        <is>
+          <t>attached</t>
+        </is>
+      </c>
+      <c r="O11" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P11" s="2" t="inlineStr">
+        <is>
+          <t>entered-with-issues</t>
+        </is>
+      </c>
+      <c r="Q11" s="2" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>O'Neal Steel - Dallas (GP)</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>15476879</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>59236</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="n">
+        <v>245.28</v>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>Success</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Finished bill (Invoice_Type 3). Header PO set=59236. Select Receipts 24374 on PO 59236. Invoice #=15476879 (exact PDF). Amount=245.28 after rounding PPV -0.04 (in-gate, not $75). Returned from Transfer AP 375 to 722. Attach status=attached. Parent Outlook Entered with issues (15476365 still HOLD).</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr"/>
+      <c r="I12" s="2" t="inlineStr"/>
+      <c r="J12" s="2" t="n">
+        <v>10179</v>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>API Agent - 9/21/26 O'Neal (722)</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>-0.04</t>
+        </is>
+      </c>
+      <c r="N12" s="2" t="inlineStr">
+        <is>
+          <t>attached</t>
+        </is>
+      </c>
+      <c r="O12" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P12" s="2" t="inlineStr">
+        <is>
+          <t>entered-with-issues</t>
+        </is>
+      </c>
+      <c r="Q12" s="2" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>O'Neal Steel - Dallas (GP)</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>15477248</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>59246</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="n">
+        <v>152.88</v>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>Success</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>Finished bill (Invoice_Type 3). Header PO set=59246. Select Receipts 24364 on PO 59246. Invoice #=15477248 (exact PDF). Amount=152.88 after rounding PPV +1.20 (in-gate, not $75). Returned from Transfer AP 375 to 722. Attach status=attached. Parent Outlook Entered with issues (15476365 still HOLD).</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr"/>
+      <c r="I13" s="2" t="inlineStr"/>
+      <c r="J13" s="2" t="n">
+        <v>10180</v>
+      </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>API Agent - 9/21/26 O'Neal (722)</t>
+        </is>
+      </c>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="inlineStr">
+        <is>
+          <t>1.20</t>
+        </is>
+      </c>
+      <c r="N13" s="2" t="inlineStr">
+        <is>
+          <t>attached</t>
+        </is>
+      </c>
+      <c r="O13" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P13" s="2" t="inlineStr">
+        <is>
+          <t>entered-with-issues</t>
+        </is>
+      </c>
+      <c r="Q13" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Q6"/>
+  <autoFilter ref="A1:Q13"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -982,7 +1495,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3">

</xml_diff>

<commit_message>
Record O'Neal finish-out: 10161 Success on 722, remaining HOLDs left.
10161 rounding PPV -0.10 then moved from Transfer AP to 722. 10079 already
Success on 375, moved to 722. 10162 still over-gate on Transfer AP.
missing_receipt 10160/10163/10175/10178 rechecked leftovers; no Select;
Anthony Comments_1. No new Aug 1+ invoices. Sheet updated.

Co-authored-by: beave89atm <beave89atm@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/runs/AP-run-2026-09-21-oneal.xlsx
+++ b/runs/AP-run-2026-09-21-oneal.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Exception counts" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'AP run'!$A$1:$Q$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'AP run'!$A$1:$Q$14</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q13"/>
+  <dimension ref="A1:Q14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -588,17 +588,17 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>category=missing_receipt; owner=Ruben Perez. HOLD (receipt): no open receipt leftover on PO 59156 for O'Neal invoice #15469453. Do not first-open guess. Ruben Perez: receiving must receive the PO so AP can Select Receipts. Comments_1 names Ruben Perez (mention-id unproven). Do not Transfer AP. Outlook AI HOLD. Flag status=entered-with-issues. Comments_1 missing_receipt status=added tab=Comments tab persisted Ruben Perez (list Comments_1 item 894, plain text (no mention-node)). User-alert/notify API not confirmed — dedicated GET comments/mentions/notifications are 404. Header Comments string is the wrong surface and is ignored. transfer_ap=False mention_id=None plain=True mail_send=False.</t>
+          <t>category=other; owner=AP. HOLD missing_receipt after leftover recheck. PO 59156 has open leftovers (24025-24029, 24052, 24053) but they do not match PDF plate lines (no Select). Comments_1 Anthony plain added (mention-id unknown). Stay 722. Do not invent Success.</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>missing_receipt</t>
+          <t>other</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>Ruben Perez</t>
+          <t>AP</t>
         </is>
       </c>
       <c r="J2" s="2" t="n">
@@ -647,11 +647,7 @@
           <t>15457895</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-28</t>
-        </is>
-      </c>
+      <c r="C3" s="2" t="inlineStr"/>
       <c r="D3" s="2" t="inlineStr">
         <is>
           <t>59068</t>
@@ -660,32 +656,24 @@
       <c r="E3" s="2" t="n">
         <v>687.26</v>
       </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>HOLD</t>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>Success</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>category=price_variance; owner=Shawn McKibben. HOLD (price-does-not-match): leftover vs invoice line is over the PPV gate. Do not Select Receipts on that line. @Shawn McKibben: purchasing must unreceive, change the PO price, and re-receive. Outlook AI HOLD. Flag status=entered-with-issues. Transfer AP status=moved batch_id=375 comment='Comments tab persisted @Shawn McKibben (list Comments_1 item 895, mention-node id 104). User-alert/notify API not confirmed — dedicated GET comments/mentions/notifications are 404. Header Comments string is the wrong surface and is ignored.' @mention=Comments tab persisted @Shawn McKibben (list Comments_1 item 895, mention-node id 104). User-alert/notify API not confirmed — dedicated GET comments/mentions/notifications are 404. Header Comments string is the wrong surface and is ignored..</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>price_variance</t>
-        </is>
-      </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>Shawn McKibben</t>
-        </is>
-      </c>
+          <t>Finished bill. Rounding/in-gate PPV -0.10 under $75. Amount=687.26. Moved to 722={'status': 'moved', 'put': 200, 'error': ''}.</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr"/>
+      <c r="I3" s="2" t="inlineStr"/>
       <c r="J3" s="2" t="n">
         <v>10161</v>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>TRANSFER AP (375)</t>
+          <t>API Agent - 9/21/26 O'Neal (722)</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
@@ -695,7 +683,7 @@
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>-0.10</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
@@ -746,17 +734,17 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>category=price_variance; owner=Shawn McKibben. HOLD (price-does-not-match): leftover vs invoice line is over the PPV gate. Do not Select Receipts on that line. @Shawn McKibben: purchasing must unreceive, change the PO price, and re-receive. Outlook AI HOLD. Flag status=entered-with-issues. Transfer AP status=moved batch_id=375 comment='Comments tab persisted @Shawn McKibben (list Comments_1 item 896, mention-node id 104). User-alert/notify API not confirmed — dedicated GET comments/mentions/notifications are 404. Header Comments string is the wrong surface and is ignored.' @mention=Comments tab persisted @Shawn McKibben (list Comments_1 item 896, mention-node id 104). User-alert/notify API not confirmed — dedicated GET comments/mentions/notifications are 404. Header Comments string is the wrong surface and is ignored..</t>
+          <t>category=missing_po; owner=Misty McCoy / Transfer AP. HOLD price_variance. PO 59070 leftovers 23581-23584 still over the $75 PPV gate (select-zero). Receipts not selected. Left on Transfer AP 375 for Treyce/Shawn. Do not invent Success.</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>price_variance</t>
+          <t>missing_po</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>Shawn McKibben</t>
+          <t>Misty McCoy / Transfer AP</t>
         </is>
       </c>
       <c r="J4" s="2" t="n">
@@ -825,17 +813,17 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>category=missing_receipt; owner=Ruben Perez. HOLD (receipt): no open receipt leftover on PO 58912 for O'Neal invoice #15464707. Do not first-open guess. Ruben Perez: receiving must receive the PO so AP can Select Receipts. Comments_1 names Ruben Perez (mention-id unproven). Do not Transfer AP. Outlook AI HOLD. Flag status=entered-with-issues. Comments_1 missing_receipt status=added tab=Comments tab persisted Ruben Perez (list Comments_1 item 897, plain text (no mention-node)). User-alert/notify API not confirmed — dedicated GET comments/mentions/notifications are 404. Header Comments string is the wrong surface and is ignored. transfer_ap=False mention_id=None plain=True mail_send=False.</t>
+          <t>category=other; owner=AP. HOLD missing_receipt after leftover recheck. PO 58912 has open leftovers (23096, 23874, 23875, 23923, 23983, 23985) but they do not match PDF lines (no Select). Comments_1 Anthony plain added. Stay 722.</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>missing_receipt</t>
+          <t>other</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>Ruben Perez</t>
+          <t>AP</t>
         </is>
       </c>
       <c r="J5" s="2" t="n">
@@ -1046,17 +1034,17 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>category=missing_receipt; owner=Anthony. HOLD (receipt): no open receipt leftover on PO 59085 for O'Neal invoice #15460995. Do not first-open guess. Anthony: receiving must receive the PO so AP can Select Receipts. Comments_1 names Anthony (mention-id unproven). Do not Transfer AP. Outlook AI HOLD. Flag status=entered-with-issues. Comments_1 missing_receipt status=added tab=Comments tab persisted Anthony (list Comments_1 item 929, plain text (no mention-node)). User-alert/notify API not confirmed — dedicated GET comments/mentions/notifications are 404. Header Comments string is the wrong surface and is ignored. transfer_ap=False mention_id=None owner=Anthony mail_send=False.</t>
+          <t>category=other; owner=AP. HOLD missing_receipt after leftover recheck. PO 59085 leftovers include 23932 (already on 10164) plus 23933/23934; none newly selectable for 15460995. Comments_1 Anthony already-on-tab. Stay 722.</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>missing_receipt</t>
+          <t>other</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>Anthony</t>
+          <t>AP</t>
         </is>
       </c>
       <c r="J8" s="2" t="n">
@@ -1267,17 +1255,17 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>category=missing_receipt; owner=Anthony. HOLD (receipt): no open receipt leftover on PO 59070 for O'Neal invoice #15476365. Do not first-open guess. Anthony: receiving must receive the PO so AP can Select Receipts. Comments_1 names Anthony (mention-id unproven). Do not Transfer AP. Outlook AI HOLD. Flag status=entered-with-issues. Comments_1 missing_receipt status=added tab=Comments tab persisted Anthony (list Comments_1 item 930, plain text (no mention-node)). User-alert/notify API not confirmed — dedicated GET comments/mentions/notifications are 404. Header Comments string is the wrong surface and is ignored. transfer_ap=False mention_id=None owner=Anthony mail_send=False.</t>
+          <t>category=other; owner=AP. HOLD missing_receipt after leftover recheck. PO 59070 leftovers 23581-23584 are the same over-gate pool as 10162; no match for $1115.68. Comments_1 Anthony already-on-tab. Stay 722. Sibling 15457895 is now Success; parent Outlook stays Entered with issues.</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>missing_receipt</t>
+          <t>other</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>Anthony</t>
+          <t>AP</t>
         </is>
       </c>
       <c r="J11" s="2" t="n">
@@ -1457,8 +1445,67 @@
       </c>
       <c r="Q13" s="2" t="inlineStr"/>
     </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>O'Neal Steel - Dallas (GP)</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>15447737</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr"/>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>58979</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="n">
+        <v>1683.01</v>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>Success</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Already-Success O'Neal on Transfer AP 375 (older header 10079). Amount=1683.01 matches verification. 4 receipts selected + 1 charge. Moved to API Agent - 9/21/26 O'Neal (722). Not a new enter. Packing slip not attached (receiving@ not reachable on this AP Graph client).</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr"/>
+      <c r="I14" s="2" t="inlineStr"/>
+      <c r="J14" s="2" t="n">
+        <v>10079</v>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>API Agent - 9/21/26 O'Neal (722)</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>1 charge already posted</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
+          <t>attached</t>
+        </is>
+      </c>
+      <c r="O14" s="2" t="inlineStr"/>
+      <c r="P14" s="2" t="inlineStr"/>
+      <c r="Q14" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Q13"/>
+  <autoFilter ref="A1:Q14"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1491,7 +1538,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>missing_receipt</t>
+          <t>other</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -1501,11 +1548,11 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>price_variance</t>
+          <t>missing_po</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Record O'Neal Fort Worth backfill: 6 unique parents moved.
13 headers had vendor PDFs. Seven sibling invoices skipped (same
message_id). Categories unchanged. No Mail.Send.

Co-authored-by: beave89atm <beave89atm@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/runs/AP-run-2026-09-21-oneal.xlsx
+++ b/runs/AP-run-2026-09-21-oneal.xlsx
@@ -634,7 +634,11 @@
           <t>entered-with-issues</t>
         </is>
       </c>
-      <c r="Q2" s="2" t="inlineStr"/>
+      <c r="Q2" s="2" t="inlineStr">
+        <is>
+          <t>NOTE-52 Fort Worth 9 - FORT WORTH ARCHIVE move=moved-fort-worth mid=AAMkAGQyODM5ZWI1LTQ0NDAtNDZiOS1hYTIzLTdjOGM3NDRlNjQ4MgBGAAAAAAAggjN_BHG4TI2Iz-JKRqfaBwDXcyWbp23lSoY0i7GBv6N_AAAAAAEMAADXcyWbp23lSoY0i7GBv6N_AAOZ_uDcAAA=.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -701,7 +705,11 @@
           <t>entered-with-issues</t>
         </is>
       </c>
-      <c r="Q3" s="2" t="inlineStr"/>
+      <c r="Q3" s="2" t="inlineStr">
+        <is>
+          <t>NOTE-52 Fort Worth 9 - FORT WORTH ARCHIVE move=moved-fort-worth mid=AAMkAGQyODM5ZWI1LTQ0NDAtNDZiOS1hYTIzLTdjOGM3NDRlNjQ4MgBGAAAAAAAggjN_BHG4TI2Iz-JKRqfaBwDXcyWbp23lSoY0i7GBv6N_AAAAAAEMAADXcyWbp23lSoY0i7GBv6N_AAOQsGW4AAA=.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -780,7 +788,11 @@
           <t>entered-with-issues</t>
         </is>
       </c>
-      <c r="Q4" s="2" t="inlineStr"/>
+      <c r="Q4" s="2" t="inlineStr">
+        <is>
+          <t>NOTE-52 Fort Worth 9 - FORT WORTH ARCHIVE move=move-skipped-already mid=AAMkAGQyODM5ZWI1LTQ0NDAtNDZiOS1hYTIzLTdjOGM3NDRlNjQ4MgBGAAAAAAAggjN_BHG4TI2Iz-JKRqfaBwDXcyWbp23lSoY0i7GBv6N_AAAAAAEMAADXcyWbp23lSoY0i7GBv6N_AAOQsGW4AAA=.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -859,7 +871,11 @@
           <t>entered-with-issues</t>
         </is>
       </c>
-      <c r="Q5" s="2" t="inlineStr"/>
+      <c r="Q5" s="2" t="inlineStr">
+        <is>
+          <t>NOTE-52 Fort Worth 9 - FORT WORTH ARCHIVE move=moved-fort-worth mid=AAMkAGQyODM5ZWI1LTQ0NDAtNDZiOS1hYTIzLTdjOGM3NDRlNjQ4MgBGAAAAAAAggjN_BHG4TI2Iz-JKRqfaBwDXcyWbp23lSoY0i7GBv6N_AAAAAAEMAADXcyWbp23lSoY0i7GBv6N_AAOVX234AAA=.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -930,7 +946,11 @@
           <t>entered-in-ai</t>
         </is>
       </c>
-      <c r="Q6" s="2" t="inlineStr"/>
+      <c r="Q6" s="2" t="inlineStr">
+        <is>
+          <t>NOTE-52 Fort Worth 9 - FORT WORTH ARCHIVE move=move-skipped-already mid=AAMkAGQyODM5ZWI1LTQ0NDAtNDZiOS1hYTIzLTdjOGM3NDRlNjQ4MgBGAAAAAAAggjN_BHG4TI2Iz-JKRqfaBwDXcyWbp23lSoY0i7GBv6N_AAAAAAEMAADXcyWbp23lSoY0i7GBv6N_AAOVX234AAA=.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1001,7 +1021,11 @@
           <t>entered-with-issues</t>
         </is>
       </c>
-      <c r="Q7" s="2" t="inlineStr"/>
+      <c r="Q7" s="2" t="inlineStr">
+        <is>
+          <t>NOTE-52 Fort Worth 9 - FORT WORTH ARCHIVE move=moved-fort-worth mid=AAMkAGQyODM5ZWI1LTQ0NDAtNDZiOS1hYTIzLTdjOGM3NDRlNjQ4MgBGAAAAAAAggjN_BHG4TI2Iz-JKRqfaBwDXcyWbp23lSoY0i7GBv6N_AAAAAAEMAADXcyWbp23lSoY0i7GBv6N_AAOQsGYLAAA=.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1080,7 +1104,11 @@
           <t>entered-with-issues</t>
         </is>
       </c>
-      <c r="Q8" s="2" t="inlineStr"/>
+      <c r="Q8" s="2" t="inlineStr">
+        <is>
+          <t>NOTE-52 Fort Worth 9 - FORT WORTH ARCHIVE move=move-skipped-already mid=AAMkAGQyODM5ZWI1LTQ0NDAtNDZiOS1hYTIzLTdjOGM3NDRlNjQ4MgBGAAAAAAAggjN_BHG4TI2Iz-JKRqfaBwDXcyWbp23lSoY0i7GBv6N_AAAAAAEMAADXcyWbp23lSoY0i7GBv6N_AAOQsGYLAAA=.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1151,7 +1179,11 @@
           <t>entered-with-issues</t>
         </is>
       </c>
-      <c r="Q9" s="2" t="inlineStr"/>
+      <c r="Q9" s="2" t="inlineStr">
+        <is>
+          <t>NOTE-52 Fort Worth 9 - FORT WORTH ARCHIVE move=move-skipped-already mid=AAMkAGQyODM5ZWI1LTQ0NDAtNDZiOS1hYTIzLTdjOGM3NDRlNjQ4MgBGAAAAAAAggjN_BHG4TI2Iz-JKRqfaBwDXcyWbp23lSoY0i7GBv6N_AAAAAAEMAADXcyWbp23lSoY0i7GBv6N_AAOQsGYLAAA=.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1222,7 +1254,11 @@
           <t>entered-with-issues</t>
         </is>
       </c>
-      <c r="Q10" s="2" t="inlineStr"/>
+      <c r="Q10" s="2" t="inlineStr">
+        <is>
+          <t>NOTE-52 Fort Worth 9 - FORT WORTH ARCHIVE move=move-skipped-already mid=AAMkAGQyODM5ZWI1LTQ0NDAtNDZiOS1hYTIzLTdjOGM3NDRlNjQ4MgBGAAAAAAAggjN_BHG4TI2Iz-JKRqfaBwDXcyWbp23lSoY0i7GBv6N_AAAAAAEMAADXcyWbp23lSoY0i7GBv6N_AAOQsGYLAAA=.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1301,7 +1337,11 @@
           <t>entered-with-issues</t>
         </is>
       </c>
-      <c r="Q11" s="2" t="inlineStr"/>
+      <c r="Q11" s="2" t="inlineStr">
+        <is>
+          <t>NOTE-52 Fort Worth 9 - FORT WORTH ARCHIVE move=moved-fort-worth mid=AAMkAGQyODM5ZWI1LTQ0NDAtNDZiOS1hYTIzLTdjOGM3NDRlNjQ4MgBGAAAAAAAggjN_BHG4TI2Iz-JKRqfaBwDXcyWbp23lSoY0i7GBv6N_AAAAAAEMAADXcyWbp23lSoY0i7GBv6N_AAOeCmQ1AAA=.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1372,7 +1412,11 @@
           <t>entered-with-issues</t>
         </is>
       </c>
-      <c r="Q12" s="2" t="inlineStr"/>
+      <c r="Q12" s="2" t="inlineStr">
+        <is>
+          <t>NOTE-52 Fort Worth 9 - FORT WORTH ARCHIVE move=move-skipped-already mid=AAMkAGQyODM5ZWI1LTQ0NDAtNDZiOS1hYTIzLTdjOGM3NDRlNjQ4MgBGAAAAAAAggjN_BHG4TI2Iz-JKRqfaBwDXcyWbp23lSoY0i7GBv6N_AAAAAAEMAADXcyWbp23lSoY0i7GBv6N_AAOeCmQ1AAA=.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1443,7 +1487,11 @@
           <t>entered-with-issues</t>
         </is>
       </c>
-      <c r="Q13" s="2" t="inlineStr"/>
+      <c r="Q13" s="2" t="inlineStr">
+        <is>
+          <t>NOTE-52 Fort Worth 9 - FORT WORTH ARCHIVE move=move-skipped-already mid=AAMkAGQyODM5ZWI1LTQ0NDAtNDZiOS1hYTIzLTdjOGM3NDRlNjQ4MgBGAAAAAAAggjN_BHG4TI2Iz-JKRqfaBwDXcyWbp23lSoY0i7GBv6N_AAAAAAEMAADXcyWbp23lSoY0i7GBv6N_AAOeCmQ1AAA=.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1502,7 +1550,11 @@
       </c>
       <c r="O14" s="2" t="inlineStr"/>
       <c r="P14" s="2" t="inlineStr"/>
-      <c r="Q14" s="2" t="inlineStr"/>
+      <c r="Q14" s="2" t="inlineStr">
+        <is>
+          <t>NOTE-52 Fort Worth 9 - FORT WORTH ARCHIVE move=moved-fort-worth mid=AAMkAGQyODM5ZWI1LTQ0NDAtNDZiOS1hYTIzLTdjOGM3NDRlNjQ4MgBGAAAAAAAggjN_BHG4TI2Iz-JKRqfaBwDXcyWbp23lSoY0i7GBv6N_AAAAAAEMAADXcyWbp23lSoY0i7GBv6N_AAOMxVrbAAA=.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:Q14"/>

</xml_diff>